<commit_message>
Dashboard 2026-09-14 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/340224629/spec-340224629.xlsx
+++ b/vse-loti/340224629/spec-340224629.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -978,18 +978,19 @@
         <v>8908617.789999999</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Источник: Документация изм.zip → Приложение №3 - Обоснование НМЦ.xls</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Источник: Документация изм.zip → Приложение №3 - Обоснование НМЦ.xls
+Документация изм.zip → Документация.docx</t>
+        </is>
+      </c>
+    </row>
     <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A17:B19"/>
+    <mergeCell ref="A18:B20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>